<commit_message>
all results from main cal, main PR and main data extract as of feb 09, 2026
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/fittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/fittingRhoResultsAll.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10,17 +10,17 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="11_B359E617CF19DF5F202E737956411E2870040D25" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{392F2AF8-C4EC-4E96-ABE9-C7432EC5B7AD}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="22" uniqueCount="10">
   <si>
     <t>model</t>
   </si>
@@ -55,8 +55,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -70,7 +70,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,12 +78,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -102,7 +104,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -253,7 +255,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -277,9 +279,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -303,7 +305,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -338,7 +340,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -356,7 +358,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -381,7 +383,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -417,59 +419,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6.85546875" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.25">
+      <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>7.6891944912210146</v>
-      </c>
-      <c r="C2">
-        <v>1.0752294085791203</v>
-      </c>
-      <c r="D2">
-        <v>4.0638467344509319</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>19.624630767628755</v>
-      </c>
-      <c r="C3">
-        <v>1.5106099978718086E-3</v>
-      </c>
-      <c r="D3">
-        <v>29.216703178032613</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="0">
+        <v>7.6891944911332928</v>
+      </c>
+      <c r="C2" s="0">
+        <v>1.075229408579305</v>
+      </c>
+      <c r="D2" s="0">
+        <v>4.0638467344371385</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.25">
+      <c r="A3" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="0">
+        <v>13.863580831435982</v>
+      </c>
+      <c r="C3" s="0">
+        <v>1.06827273026128</v>
+      </c>
+      <c r="D3" s="0">
+        <v>3.293808272865741</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -483,7 +485,7 @@
         <v>31.832079132489156</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -497,7 +499,7 @@
         <v>3.2938082729237652</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -511,7 +513,7 @@
         <v>4.4976101340301264</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
main Cal with rho ref using PR at T_MFM, cal curve with all Qs and high pressure (He, H2, CO2), fitting params saved as well as plots
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/fittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/fittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="24" uniqueCount="12">
   <si>
     <t>model</t>
   </si>
@@ -31,6 +31,24 @@
   </si>
   <si>
     <t>RMSE</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>Q10</t>
+  </si>
+  <si>
+    <t>QAll</t>
   </si>
 </sst>
 </file>
@@ -76,18 +94,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6.85546875" customWidth="true"/>
-    <col min="2" max="2" width="11.7109375" customWidth="true"/>
-    <col min="3" max="3" width="11.7109375" customWidth="true"/>
-    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="1" max="1" width="4.33203125" customWidth="true"/>
+    <col min="2" max="2" width="11.5546875" customWidth="true"/>
+    <col min="3" max="3" width="11.5546875" customWidth="true"/>
+    <col min="4" max="4" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>3</v>
@@ -101,30 +119,72 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B2" s="0">
-        <v>7.6891944911332928</v>
+        <v>10.610219799565622</v>
       </c>
       <c r="C2" s="0">
-        <v>1.075229408579305</v>
+        <v>1.0738303883336688</v>
       </c>
       <c r="D2" s="0">
-        <v>4.0638467344371385</v>
+        <v>2.2566874638904966</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B3" s="0">
-        <v>13.863580831435982</v>
+        <v>13.126555770707963</v>
       </c>
       <c r="C3" s="0">
-        <v>1.06827273026128</v>
+        <v>1.0767697251626287</v>
       </c>
       <c r="D3" s="0">
-        <v>3.293808272865741</v>
+        <v>1.2385353367296099</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="0">
+        <v>15.320883900505974</v>
+      </c>
+      <c r="C4" s="0">
+        <v>1.075073428886018</v>
+      </c>
+      <c r="D4" s="0">
+        <v>1.0166706989085621</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="0">
+        <v>14.041943772708919</v>
+      </c>
+      <c r="C5" s="0">
+        <v>1.0801434655138764</v>
+      </c>
+      <c r="D5" s="0">
+        <v>2.1962298394769211</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="0">
+        <v>13.527936420493747</v>
+      </c>
+      <c r="C6" s="0">
+        <v>1.0740311270539915</v>
+      </c>
+      <c r="D6" s="0">
+        <v>2.7030797604930483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes to capture Q_effect but to be removed since it does not solve the issue of C error at higher concentration of H2
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/fittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/fittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="78" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="114" uniqueCount="12">
   <si>
     <t>model</t>
   </si>
@@ -97,10 +97,10 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.33203125" customWidth="true"/>
-    <col min="2" max="2" width="11.5546875" customWidth="true"/>
-    <col min="3" max="3" width="11.5546875" customWidth="true"/>
-    <col min="4" max="4" width="11.5546875" customWidth="true"/>
+    <col min="1" max="1" width="4.5703125" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>